<commit_message>
feat(playground): SNR<->RSSI link budget, PER-chart wanted-SNR table, rename architecture
- Live PER chart: 'Wanted SNR' slider (synced) + per-MCS PER/SR table under the graph

- B2 PER model: SNR->RSSI worked example table (NF 4 + 8 dB margin) vs RSSI->MCS SAS model

- Decisions: document the RSSI<->SNR link budget + derived 8 dB implementation margin

- XLSX 'RSSI to SNR' sheet reformatted as a per-BW table; dual SNR/RSSI chart axis; x/square/circle markers

- Rename tlc_sim_architecture_old.html -> tlc_sim_architecture.html; fix iframe loading

- Add reference lab TVA SCD sum JSONs (PERModel/RefTVA) + PER model html/md doc
</commit_message>
<xml_diff>
--- a/PERModel/RSSI_to_MCS_and_TpT_Mapping.xlsx
+++ b/PERModel/RSSI_to_MCS_and_TpT_Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://intel-my.sharepoint.com/personal/efrat_isack_intel_com/Documents/Desktop/Efrat/TLC_Sim/PERModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_113BDC59A7D19EA1F6CF7A896053802B3E124F51" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10A9FD46-8582-41B2-9B2A-CAECD658D49A}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="11_113BDC59A7D19EA1F6CF7A896053802B3E124F51" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2BC3BE9-05D5-42B0-9030-8B494A03579E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="9" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,25 @@
     <sheet name="UHR 160MHz" sheetId="21" r:id="rId21"/>
     <sheet name="UHR 320MHz" sheetId="22" r:id="rId22"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="105">
   <si>
     <t>RSSI to MCS and TpT Mapping</t>
   </si>
@@ -340,11 +353,32 @@
   <si>
     <t>c</t>
   </si>
+  <si>
+    <t>bw</t>
+  </si>
+  <si>
+    <t>Estimated RSSI</t>
+  </si>
+  <si>
+    <t>required dbm for MCS13 from RSSI model</t>
+  </si>
+  <si>
+    <t>require SNR for 10% per EHT 0.8us GI 320MHZ, from philip PER model</t>
+  </si>
+  <si>
+    <t>Intel Noise figure</t>
+  </si>
+  <si>
+    <t>Calc Noise Floor</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -460,7 +494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -484,6 +518,21 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,6 +548,76 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{659F7F7C-F072-9E36-A6CA-5A9D28E6EA82}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="698500" y="6292850"/>
+          <a:ext cx="7213600" cy="717550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4752,7 +4871,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:T33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -5082,7 +5201,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>-64.5</v>
       </c>
@@ -5108,7 +5227,7 @@
         <v>1960</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>-62.5</v>
       </c>
@@ -5134,7 +5253,7 @@
         <v>2205</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>-61</v>
       </c>
@@ -5160,7 +5279,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>-57</v>
       </c>
@@ -5186,7 +5305,7 @@
         <v>2940</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>-55</v>
       </c>
@@ -5212,7 +5331,7 @@
         <v>3266.6</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>-50.5</v>
       </c>
@@ -5238,7 +5357,7 @@
         <v>3675</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>-47.5</v>
       </c>
@@ -5264,7 +5383,7 @@
         <v>4083.2</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>-43</v>
       </c>
@@ -5290,7 +5409,7 @@
         <v>4410</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>-40</v>
       </c>
@@ -5314,6 +5433,71 @@
       </c>
       <c r="H25" s="8">
         <v>4900</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A28" s="14">
+        <v>-40</v>
+      </c>
+      <c r="B28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A29" s="15">
+        <f>37</f>
+        <v>37</v>
+      </c>
+      <c r="B29" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A30" s="16">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A31" s="16">
+        <v>320</v>
+      </c>
+      <c r="B31" t="s">
+        <v>99</v>
+      </c>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
+      <c r="O31" s="13"/>
+      <c r="P31" s="13"/>
+      <c r="Q31" s="13"/>
+      <c r="R31" s="13"/>
+      <c r="S31" s="13"/>
+      <c r="T31" s="13"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A32" s="17">
+        <f>10*LOG10(A31*1000000)-174+A30</f>
+        <v>-79.948500216800937</v>
+      </c>
+      <c r="B32" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="17">
+        <f>A32+A29</f>
+        <v>-42.948500216800937</v>
+      </c>
+      <c r="B33" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -5322,6 +5506,7 @@
     <mergeCell ref="F5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>